<commit_message>
feat(EVERGREEN_LOGISTICS): 新增 VAT 單一總額合成列 + 含稅總額稽核
VAT 只有整張帳單一個總額 (不是逐筆列出)，獨立成一筆 description=None/
amount=None/vat=稅額 的合成列，跟 KUEHNE_NAGEL/TRANS_DAYA_PRIMA/APL 同一
套慣例 (只有一筆費用明細時 Description 沿用該筆描述，兩筆以上留空)。
掛上含稅總額稽核 (未稅加總 + VAT = 帳單最下方那行含稅總額)。Shipper
欄位這兩個樣本的正確答案都是空白，不需要額外擷取規則，缺漏會自動補
N/A。

新增第 2 組回歸測試樣本 (00048623)。兩份新範本各有一個日期格式跟系統
現有慣例不一致 (Arrive Date 變回斜線格式 '2026/07/01'、INVOICE DATE
其中一筆填成純文字 '05.06.2026' 而不是 Excel 日期型態)，已跟使用者
確認「全部日期都要用 DD Mon YYYY 英文縮寫格式、INVOICE DATE 要維持
Excel 日期型態」，程式碼不用改，是範本本身的格式問題，已在收錄回歸
樣本時連同修正。run_regression.py (EVERGREEN_LOGISTICS) 100% 通過，
兩個 Streamlit App 開機測試正常。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JhL7qxuxZLsZyoRKZr1of6
</commit_message>
<xml_diff>
--- a/test_samples/EVERGREEN_LOGISTICS/sample1_ref.xlsx
+++ b/test_samples/EVERGREEN_LOGISTICS/sample1_ref.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15465" yWindow="-13620" windowWidth="24240" windowHeight="13020" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="10590" yWindow="4545" windowWidth="21660" windowHeight="14550" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
@@ -498,24 +498,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="16.453125" customWidth="1" style="8" min="1" max="1"/>
-    <col width="15.7265625" customWidth="1" style="8" min="2" max="2"/>
-    <col width="34.54296875" customWidth="1" style="8" min="3" max="3"/>
+    <col width="16.5" customWidth="1" style="8" min="1" max="1"/>
+    <col width="15.75" customWidth="1" style="8" min="2" max="2"/>
+    <col width="34.5" customWidth="1" style="8" min="3" max="3"/>
     <col width="26" customWidth="1" style="8" min="4" max="4"/>
-    <col width="25.453125" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
-    <col width="17.90625" customWidth="1" style="8" min="6" max="6"/>
-    <col width="29.26953125" customWidth="1" style="8" min="7" max="7"/>
-    <col width="13.7265625" customWidth="1" style="8" min="8" max="9"/>
-    <col width="20.54296875" customWidth="1" style="8" min="10" max="10"/>
-    <col width="20" customWidth="1" style="8" min="11" max="11"/>
-    <col width="16.90625" bestFit="1" customWidth="1" style="8" min="12" max="12"/>
-    <col width="18.6328125" bestFit="1" customWidth="1" style="8" min="13" max="13"/>
-    <col width="16.36328125" customWidth="1" style="8" min="14" max="14"/>
-    <col width="20.6328125" customWidth="1" style="8" min="15" max="15"/>
-    <col width="15.08984375" bestFit="1" customWidth="1" style="8" min="16" max="16"/>
+    <col width="25.5" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
+    <col width="17.875" customWidth="1" style="8" min="6" max="7"/>
+    <col width="29.25" customWidth="1" style="8" min="8" max="8"/>
+    <col width="13.75" customWidth="1" style="8" min="9" max="10"/>
+    <col width="20.5" customWidth="1" style="8" min="11" max="11"/>
+    <col width="20" customWidth="1" style="8" min="12" max="12"/>
+    <col width="16.875" bestFit="1" customWidth="1" style="8" min="13" max="13"/>
+    <col width="18.625" bestFit="1" customWidth="1" style="8" min="14" max="14"/>
+    <col width="16.375" customWidth="1" style="8" min="15" max="15"/>
+    <col width="20.625" customWidth="1" style="8" min="16" max="16"/>
+    <col width="15.125" bestFit="1" customWidth="1" style="8" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customFormat="1" customHeight="1" s="6">
@@ -557,61 +557,72 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Order No.</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Arrive Date
 到達日</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>on board date
 開船日</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>B/L NO.
 提單號碼</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>MBL NO.
 主提單號碼</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Port of Loading
 啟運港</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Port of discharge
 目的港</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Volume
 材積</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Vessel
 船名</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Container no.
 貨櫃號碼</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Shipper
+出貨方</t>
         </is>
       </c>
     </row>
@@ -642,54 +653,59 @@
       <c r="F2" s="4" t="n">
         <v>2668350</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>RWRD501600002926</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>KMTCPUSK052666</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>KMSU 2606S</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>KMTU9431774</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -720,54 +736,59 @@
       <c r="F3" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>RWRD501600002926</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>KMTCPUSK052666</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>KMSU 2606S</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>KMTU9431774</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -798,54 +819,59 @@
       <c r="F4" s="4" t="n">
         <v>444725</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>RWRD501600002926</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>KMTCPUSK052666</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>KMSU 2606S</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>KMTU9431774</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -876,54 +902,59 @@
       <c r="F5" s="4" t="n">
         <v>11562850</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>RWRD501600002926</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>KMTCPUSK052666</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>KMSU 2606S</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>KMTU9431774</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -954,148 +985,224 @@
       <c r="F6" s="4" t="n">
         <v>2864029</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>RWRD501600002926</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>KMTCPUSK052666</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>KMSU 2606S</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>KMTU9431774</t>
         </is>
       </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="1" s="4">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="A7" s="7" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>00049334</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>P.T. EVERGREEN LOGISTICS INDONESIA</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>PT. POU YUEN INDONESIA</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>192939</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>01 Jul 2026</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>RWRD501600002926</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>KMTCPUSK052666</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>JAKARTA</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>KMSU 2606S</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>KMTU9431774</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="1" s="4">
       <c r="A8" s="3" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="H8" s="5" t="n"/>
       <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" customFormat="1" s="4">
       <c r="A9" s="3" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="H9" s="5" t="n"/>
       <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" customFormat="1" s="4">
       <c r="A10" s="3" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="H10" s="5" t="n"/>
       <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" customFormat="1" s="4">
       <c r="A11" s="3" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="H11" s="5" t="n"/>
       <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
     </row>
     <row r="12" customFormat="1" s="4">
       <c r="A12" s="3" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="H12" s="5" t="n"/>
       <c r="I12" s="3" t="n"/>
-      <c r="Q12" s="6" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="R12" s="6" t="n"/>
     </row>
     <row r="13" customFormat="1" s="4">
       <c r="A13" s="3" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="3" t="n"/>
+      <c r="H13" s="5" t="n"/>
       <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
     </row>
     <row r="14" customFormat="1" s="4">
       <c r="A14" s="3" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="H14" s="5" t="n"/>
       <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" customFormat="1" s="4">
       <c r="A15" s="3" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="H15" s="5" t="n"/>
       <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
     </row>
     <row r="16" customFormat="1" s="4">
       <c r="A16" s="3" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="3" t="n"/>
+      <c r="H16" s="5" t="n"/>
       <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
     </row>
     <row r="17" customFormat="1" s="4">
       <c r="A17" s="3" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="3" t="n"/>
+      <c r="H17" s="5" t="n"/>
       <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
     </row>
     <row r="18" customFormat="1" s="4">
       <c r="A18" s="3" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="3" t="n"/>
+      <c r="H18" s="5" t="n"/>
       <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
     </row>
     <row r="19" customFormat="1" s="4">
       <c r="A19" s="3" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="3" t="n"/>
+      <c r="H19" s="5" t="n"/>
       <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
     </row>
     <row r="20" customFormat="1" s="4">
       <c r="A20" s="3" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="3" t="n"/>
+      <c r="H20" s="5" t="n"/>
       <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
     </row>
     <row r="21" customFormat="1" s="4">
       <c r="A21" s="3" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="3" t="n"/>
+      <c r="H21" s="5" t="n"/>
       <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>